<commit_message>
Price Shopee rows per original package.
Shopee Unit Price is Total Penjualan Per Produk times bobot divided by the Jubelio Qty before qty_bundle. The column is labeled Unit Price in the table and Excel export. Accurate unitPrice stays the price per output quantity.

Co-authored-by: support <support@mataharilabs.com>
</commit_message>
<xml_diff>
--- a/samples/rapi-penjualan-2026-10-26-lintas-sby-jkt.xlsx
+++ b/samples/rapi-penjualan-2026-10-26-lintas-sby-jkt.xlsx
@@ -1441,7 +1441,7 @@
         <v>2</v>
       </c>
       <c r="E39" s="1" t="n">
-        <v>360000</v>
+        <v>180000</v>
       </c>
       <c r="F39" s="1" t="n">
         <v>0</v>
@@ -2351,7 +2351,7 @@
         <v>8</v>
       </c>
       <c r="E74" s="1" t="n">
-        <v>35500</v>
+        <v>17750</v>
       </c>
       <c r="F74" s="1" t="n">
         <v>2000</v>
@@ -4249,7 +4249,7 @@
         <v>8</v>
       </c>
       <c r="E147" s="1" t="n">
-        <v>29000</v>
+        <v>14500</v>
       </c>
       <c r="F147" s="1" t="n">
         <v>0</v>
@@ -5029,7 +5029,7 @@
         <v>8</v>
       </c>
       <c r="E177" s="1" t="n">
-        <v>35500</v>
+        <v>17750</v>
       </c>
       <c r="F177" s="1" t="n">
         <v>250</v>
@@ -6537,7 +6537,7 @@
         <v>20</v>
       </c>
       <c r="E235" s="1" t="n">
-        <v>11400</v>
+        <v>5700</v>
       </c>
       <c r="F235" s="1" t="n">
         <v>0</v>
@@ -6667,7 +6667,7 @@
         <v>8</v>
       </c>
       <c r="E240" s="1" t="n">
-        <v>25950</v>
+        <v>12975</v>
       </c>
       <c r="F240" s="1" t="n">
         <v>150</v>
@@ -6953,7 +6953,7 @@
         <v>8</v>
       </c>
       <c r="E251" s="1" t="n">
-        <v>35500</v>
+        <v>17750</v>
       </c>
       <c r="F251" s="1" t="n">
         <v>0</v>
@@ -7577,7 +7577,7 @@
         <v>3</v>
       </c>
       <c r="E275" s="1" t="n">
-        <v>294000</v>
+        <v>98000</v>
       </c>
       <c r="F275" s="1" t="n">
         <v>15000</v>
@@ -10463,7 +10463,7 @@
         <v>60</v>
       </c>
       <c r="E386" s="1" t="n">
-        <v>33000</v>
+        <v>5500</v>
       </c>
       <c r="F386" s="1" t="n">
         <v>0</v>
@@ -11139,7 +11139,7 @@
         <v>24</v>
       </c>
       <c r="E412" s="1" t="n">
-        <v>34833.33333333333</v>
+        <v>17416.66666666666</v>
       </c>
       <c r="F412" s="1" t="n">
         <v>1250</v>
@@ -11893,7 +11893,7 @@
         <v>3</v>
       </c>
       <c r="E441" s="1" t="n">
-        <v>63000</v>
+        <v>21000</v>
       </c>
       <c r="F441" s="1" t="n">
         <v>600</v>

</xml_diff>

<commit_message>
Make Total Diskon a per-package amount on every channel.
Divide the existing discount by the original Jubelio Qty. Non-Shopee Unit Price is unchanged. Accurate itemCashDiscount stays the line discount.

Co-authored-by: support <support@mataharilabs.com>
</commit_message>
<xml_diff>
--- a/samples/rapi-penjualan-2026-10-26-lintas-sby-jkt.xlsx
+++ b/samples/rapi-penjualan-2026-10-26-lintas-sby-jkt.xlsx
@@ -450,7 +450,7 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>Harga Jual</t>
+          <t>Unit Price</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
@@ -2354,7 +2354,7 @@
         <v>17750</v>
       </c>
       <c r="F74" s="1" t="n">
-        <v>2000</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="75">
@@ -5032,7 +5032,7 @@
         <v>17750</v>
       </c>
       <c r="F177" s="1" t="n">
-        <v>250</v>
+        <v>125</v>
       </c>
     </row>
     <row r="178">
@@ -6670,7 +6670,7 @@
         <v>12975</v>
       </c>
       <c r="F240" s="1" t="n">
-        <v>150</v>
+        <v>75</v>
       </c>
     </row>
     <row r="241">
@@ -7580,7 +7580,7 @@
         <v>98000</v>
       </c>
       <c r="F275" s="1" t="n">
-        <v>15000</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="276">
@@ -11142,7 +11142,7 @@
         <v>17416.66666666666</v>
       </c>
       <c r="F412" s="1" t="n">
-        <v>1250</v>
+        <v>625</v>
       </c>
     </row>
     <row r="413">
@@ -11896,7 +11896,7 @@
         <v>21000</v>
       </c>
       <c r="F441" s="1" t="n">
-        <v>600</v>
+        <v>200</v>
       </c>
     </row>
     <row r="442">

</xml_diff>